<commit_message>
Ajout couverture coiale + narratif + exemples 83477ca7dfa1ca6c847db3203fad7426df761851
</commit_message>
<xml_diff>
--- a/nmoreau/ig/CodeSystem-encounter-class-code-system.xlsx
+++ b/nmoreau/ig/CodeSystem-encounter-class-code-system.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop-sante.fr/fhir/CodeSystem/encounter-class-code-system</t>
+    <t>http://hl7.fr/fhir/fr/preadmission/CodeSystem/encounter-class-code-system</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-18T09:05:02+00:00</t>
+    <t>2025-04-24T12:12:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>